<commit_message>
Weekly audit for any team: three questions, team files, interactive HTML
- SKILL.md is general: weekly audit (were tasks created, company links, workflow changes), setup step, how to set up a new team; CS Ops rules removed
- Team settings come from audits/<team>-workflow-audit/team-rules.md (json block); teams.json removed
- fetch.py --weekly, weekly.py (three questions), weekly_html.py (tabs, task-type dropdown, facility search)
- master.py compares live workflows with the master rules file
- CS Ops: F-05 Reminders added as known issue and Waiting on Cherine item; branch reasons and decision owner in settings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
+++ b/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -485,6 +485,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -608,48 +609,72 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Known issue F-08</t>
+          <t>Known issue F-05</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>"Create Tasks | Respond to reviews at Storage Reach" didn't come back from the API. It's a User workflow, which may be why.</t>
+          <t>R+S - Reminders: Respond within 1 day to external emails (1689020435) creates no tasks: it only branches and waits, then loops back.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Known issue OFF-5</t>
+          <t>Known issue F-08</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>5 workflows are switched off. That's expected unless WLS says otherwise.</t>
+          <t>"Create Tasks | Respond to reviews at Storage Reach" didn't come back from the API. It's a User workflow, which may be why.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Not in this file</t>
+          <t>Known issue OFF-5</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Create Tasks | Respond to reviews at Storage Reach (known issue F-08): its settings could not be read.</t>
+          <t>5 workflows are switched off. That's expected unless WLS says otherwise.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Not in this file</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Create Tasks | Respond to reviews at Storage Reach (known issue F-08): its settings could not be read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Change log</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>2026-10-07: file created.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07: added known issue F-05 (Reminders creates no tasks), confirmed by WLS. No workflow rows changed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CS Ops: apply Cherine's answers (2026-10-08)
- Master rules file updated from the live workflows for the planned changes only: 47 empty branches and Storage Reach's Enterprise branch deleted, Weekly calls revision; R+S - Reminders removed (deleted). One log line per workflow. Weekly KPI review stays ON.
- team-rules.md: Waiting on Cherine 4, 5, 6 and known issues F-05, BOG-Q closed; items 1 and 2 reworded; Tier 2 - L1 with no OM in Sentiment is excluded by rule
- weekly.py: branch reasons can check company values and workflows, so Tier 1 facilities with an SM keep the Tier 1 SM gap reason; clearer message when a task was moved by a workflow that no longer exists
- master.py: remove command for deleted workflows

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
+++ b/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Settings (for scripts)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Rules'!$A$1:$S$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master Rules'!$A$1:$S$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -485,7 +485,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -675,6 +674,234 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>2026-10-07: added known issue F-05 (Reminders creates no tasks), confirmed by WLS. No workflow rows changed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1770961042. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start). Revision 54 -&gt; 55.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1770960918. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 2 - L1" (start), "Tier 2 - L2" (start), "Tier 3" (start), "SOA" (start), "T1 SM" (under "Tier 1"). Revision 34 -&gt; 36.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1838568063. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start), "T1 SM" (under "Tier 1"). Revision 30 -&gt; 32.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682560327. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start), "T1 SM" (under "Tier 1"). Revision 103 -&gt; 105.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682542430. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 2 - L2" (start), "Tier 3" (start), "SOA" (start). Revision 140 -&gt; 141.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1868006300. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Enterprise" (start), "Tier 1" (start), "Tier 2 - L1" (start), "SOA" (start). Revision 13 -&gt; 14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1838565797. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start). Revision 35 -&gt; 36.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682548292. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start). Revision 90 -&gt; 91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682559152. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 2 - L2" (start), "Tier 3" (start), "SOA" (start), "T1 SM" (under "Tier 1"), "Tier 2 - L1 SM" (under "Tier 2 - L1"). Revision 142 -&gt; 145.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1868006311. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Enterprise" (start), "Tier 1" (start), "Tier 2 - L1" (start), "SOA" (start). Revision 14 -&gt; 15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1838565644. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start), "T1 SM" (under "Tier 1"). Revision 39 -&gt; 43. Also the revision change from 39 to 41 seen on 2026-10-07, confirmed as planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1838568062. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start), "T1 SM" (under "Tier 1"). Revision 28 -&gt; 32. Its on/off state is not part of this update: it is ON, as recorded; switching it off was not confirmed (Waiting on Cherine item 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1688964146. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 1" (start), "Tier 2 - L1" (start), "Tier 2 - L2" (start), "Tier 3" (start). Revision 75 -&gt; 76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1688976731. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start), "T1 SM" (under "Tier 1"). Revision 83 -&gt; 85.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682545542. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 3" (start), "SOA" (start). Revision 65 -&gt; 66.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682101413. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "SOA" (start). Revision 108 -&gt; 109.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1682549368. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 2 - L2" (start), "SOA" (start). Revision 141 -&gt; 142.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1697631666. Planned (confirmed by WLS on 2026-10-08): deleted branches with no task: "Tier 2 - L2" (start), "Is OM" (under "Tier 1"), "Enterprise OM" (under "Enterprise"), "Enterprise SM" (under "Enterprise"), "Enterprise" (start; it held only empty branches). Revision 21 -&gt; 23. The "Enterprise" branch held only the empty "Enterprise OM" / "Enterprise SM" branches; no task was lost (confirmed as planned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: removed R+S - Reminders: Respond within 1 day to external emails (1689020435). Deleted in HubSpot on purpose (confirmed by WLS on 2026-10-08); the API now returns 404. Closes known issue F-05 and Waiting on Cherine item 4.</t>
         </is>
       </c>
     </row>
@@ -689,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S24"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -858,14 +1085,13 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "Tier 1 OM" if Operations Manager is known; "Tier 1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L2 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -908,12 +1134,12 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:23:05 UTC</t>
+          <t>2026-10-08 08:15:10 UTC</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr"/>
@@ -966,16 +1192,11 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name does_not_contain SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name does_not_contain SOA; "SOA" if Company name starts with SOA -; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
-"Tier 2 - L1": ends with no task
-"Tier 2 - L2": ends with no task
-"Tier 3": ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1013,12 +1234,12 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>36</t>
         </is>
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:18:49 UTC</t>
+          <t>2026-10-08 08:16:15 UTC</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr"/>
@@ -1071,15 +1292,13 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1121,12 +1340,12 @@
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:13:17 UTC</t>
+          <t>2026-10-08 08:17:04 UTC</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr"/>
@@ -1179,15 +1398,13 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 At "Tier 2 - L1": "T2-L1 OM" if Operations Manager is known; "T2-L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1229,12 +1446,12 @@
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>105</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 10:36:59 UTC</t>
+          <t>2026-10-08 08:22:28 UTC</t>
         </is>
       </c>
       <c r="S5" s="5" t="inlineStr"/>
@@ -1394,16 +1611,13 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"Tier 2 - L2": ends with no task
-"Tier 3": ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1444,12 +1658,12 @@
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 11:01:53 UTC</t>
+          <t>2026-10-08 08:19:10 UTC</t>
         </is>
       </c>
       <c r="S7" s="5" t="inlineStr"/>
@@ -1502,11 +1716,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
-"Enterprise": ends with no task
-"Tier 1": ends with no task
-"Tier 2 - L1": ends with no task
-"SOA": ends with no task
+          <t>At (start): "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 None met: ends with no task</t>
         </is>
       </c>
@@ -1543,12 +1753,12 @@
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 10:58:00 UTC</t>
+          <t>2026-10-08 08:19:36 UTC</t>
         </is>
       </c>
       <c r="S8" s="5" t="inlineStr"/>
@@ -1601,14 +1811,13 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1650,12 +1859,12 @@
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>36</t>
         </is>
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 10:54:11 UTC</t>
+          <t>2026-10-08 08:20:19 UTC</t>
         </is>
       </c>
       <c r="S9" s="5" t="inlineStr"/>
@@ -1708,14 +1917,13 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "T2 - L1 OM" if Operations Manager is known; "T2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1758,12 +1966,12 @@
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:24:49 UTC</t>
+          <t>2026-10-08 08:14:43 UTC</t>
         </is>
       </c>
       <c r="S10" s="5" t="inlineStr"/>
@@ -1816,18 +2024,13 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
-At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
+At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
-"Tier 2 - L1" &gt; "Tier 2 - L1 SM": ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"Tier 2 - L2": ends with no task
-"Tier 3": ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -1866,12 +2069,12 @@
       </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>145</t>
         </is>
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:10:58 UTC</t>
+          <t>2026-10-08 08:17:52 UTC</t>
         </is>
       </c>
       <c r="S11" s="5" t="inlineStr"/>
@@ -1924,11 +2127,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
-"Enterprise": ends with no task
-"Tier 1": ends with no task
-"Tier 2 - L1": ends with no task
-"SOA": ends with no task
+          <t>At (start): "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 None met: ends with no task</t>
         </is>
       </c>
@@ -1965,12 +2164,12 @@
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:06:35 UTC</t>
+          <t>2026-10-08 08:18:24 UTC</t>
         </is>
       </c>
       <c r="S12" s="5" t="inlineStr"/>
@@ -2023,15 +2222,13 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -2073,12 +2270,12 @@
       </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>43</t>
         </is>
       </c>
       <c r="R13" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:15:48 UTC</t>
+          <t>2026-10-08 08:12:55 UTC</t>
         </is>
       </c>
       <c r="S13" s="5" t="inlineStr"/>
@@ -2131,15 +2328,13 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -2181,12 +2376,12 @@
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>32</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:17:37 UTC</t>
+          <t>2026-10-08 08:12:20 UTC</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr"/>
@@ -2239,13 +2434,9 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1": ends with no task
-"Tier 2 - L1": ends with no task
-"Tier 2 - L2": ends with no task
-"Tier 3": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -2283,12 +2474,12 @@
       </c>
       <c r="Q15" s="5" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:26:04 UTC</t>
+          <t>2026-10-08 08:14:12 UTC</t>
         </is>
       </c>
       <c r="S15" s="5" t="inlineStr"/>
@@ -2448,15 +2639,13 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
+At "Tier 1": "T1 OM" if Operations Manager is known; otherwise end
 At "Tier 2 - L1": "Tier 2 - L1 OM" if Operations Manager is known; "Tier 2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "T1 SM": ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
@@ -2498,12 +2687,12 @@
       </c>
       <c r="Q17" s="5" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>85</t>
         </is>
       </c>
       <c r="R17" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:29:34 UTC</t>
+          <t>2026-10-08 08:13:30 UTC</t>
         </is>
       </c>
       <c r="S17" s="5" t="inlineStr"/>
@@ -2511,12 +2700,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>R+S - Reminders: Respond within 1 day to external emails</t>
+          <t>T1 SM SOA | R+S - Execute Monthly Walk Through - BOG</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>1689020435</t>
+          <t>1688833555</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2531,82 +2720,73 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Meant to remind managers to answer external emails within 1 day. Today it only branches and waits; it creates nothing (finding F-05).</t>
+          <t>Monthly (day 1): gives SOA facilities a 'Execute Monthly Walk Through' task for the Site Manager. Other facilities get nothing from it.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center) AND an associated record where hs_email_direction is any of INCOMING_EMAIL</t>
+          <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
+          <t>Re-checked every month on day(s) 1 at 00:00</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>At (start): "SOA" if Company name starts with SOA - ; otherwise end
+None met: ends with no task</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>"SOA": "R+S - Execute Monthly Walk Through" | type TODO | priority NONE | owner record's Site Manager | due 2 business day(s) after creation at 08:00 | queue Ops Tasks (13519269) | links Company = enrolled record | description 139 chars | description id 863f62f78287</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>At (start): "SLA not met" if Last Contacted (Ticket Note) is before; otherwise end
-At "SLA not met": "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
-At "SLA not met" &gt; "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
-"SLA not met" &gt; "Tier 1" &gt; "T1 OM": ends with no task
-"SLA not met" &gt; "Tier 1" &gt; "T1 SM": ends with no task
-"SLA not met" &gt; "Tier 1" &gt; None met: ends with no task
-"SLA not met" &gt; "Tier 2": ends with no task
-"SLA not met" &gt; "Tier 3": ends with no task
-"SLA not met" &gt; "SOA": ends with no task
-"SLA not met" &gt; None met: ends with no task
-None met: ends with no task</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>(start): Delay - 1440 minutes</t>
-        </is>
-      </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>4 (3 If/then branch, 1 Delay)</t>
+          <t>2 (1 If/then branch, 1 Create task)</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>Branches on: Customer Tier, Company name, Operations Manager, Site Manager, Last Contacted (Ticket Note)</t>
+          <t>Creates task(s): "R+S - Execute Monthly Walk Through". Branches on: Company name</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
-          <t>None (creates no tasks)</t>
+          <t>Execute Monthly Walk Through</t>
         </is>
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>n/a (no task actions)</t>
+          <t>Ops Tasks (13519269) on all 1 task action(s)</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>23</t>
         </is>
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
-          <t>2026-10-06 13:26:35 UTC</t>
+          <t>2026-10-06 13:28:00 UTC</t>
         </is>
       </c>
       <c r="S18" s="5" t="inlineStr"/>
@@ -2614,12 +2794,12 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>T1 SM SOA | R+S - Execute Monthly Walk Through - BOG</t>
+          <t>Create Tasks | Playbook Review/Maintenance T1 OM</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>1688833555</t>
+          <t>1682545542</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -2629,12 +2809,12 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Monthly (day 1): gives SOA facilities a 'Execute Monthly Walk Through' task for the Site Manager. Other facilities get nothing from it.</t>
+          <t>Switched off. Older Playbook Review/Maintenance workflow for Tier 1 OMs (replaced by Playbook Review/Maintenance).</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -2644,7 +2824,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Re-checked every month on day(s) 1 at 00:00</t>
+          <t>Re-checked every month on day(s) 1 at 10:00</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -2654,118 +2834,22 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>record is in list 4291 "Exclude from Ops tasks"</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>At (start): "SOA" if Company name starts with SOA - ; otherwise end
-None met: ends with no task</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>"SOA": "R+S - Execute Monthly Walk Through" | type TODO | priority NONE | owner record's Site Manager | due 2 business day(s) after creation at 08:00 | queue Ops Tasks (13519269) | links Company = enrolled record | description 139 chars | description id 863f62f78287</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
-        <is>
-          <t>2 (1 If/then branch, 1 Create task)</t>
-        </is>
-      </c>
-      <c r="N19" s="5" t="inlineStr">
-        <is>
-          <t>Creates task(s): "R+S - Execute Monthly Walk Through". Branches on: Company name</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="inlineStr">
-        <is>
-          <t>Execute Monthly Walk Through</t>
-        </is>
-      </c>
-      <c r="P19" s="5" t="inlineStr">
-        <is>
-          <t>Ops Tasks (13519269) on all 1 task action(s)</t>
-        </is>
-      </c>
-      <c r="Q19" s="5" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="R19" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-06 13:28:00 UTC</t>
-        </is>
-      </c>
-      <c r="S19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Create Tasks | Playbook Review/Maintenance T1 OM</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>1682545542</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Switched off. Older Playbook Review/Maintenance workflow for Tier 1 OMs (replaced by Playbook Review/Maintenance).</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Re-checked every month on day(s) 1 at 10:00</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>record is in list 4291 "Exclude from Ops tasks"</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 -L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 -L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA; otherwise end
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 -L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 -L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1  SM" if Site Manager is known; otherwise end
 At "Tier 2 -L1": "T2 - L1 OM" if Operations Manager is known; "T2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 -L1" &gt; None met: ends with no task
-"Tier 3": ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>"Enterprise" &gt; "Enterprise OM": "R+S - Playbook Review/Maintenance" | type TODO | priority NONE | owner record's Operations Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 171 chars | description id 0cc8b2ca0aad
 "Enterprise" &gt; "Enterprise SM": "R+S - Playbook Review/Maintenance" | type TODO | priority NONE | owner record's Site Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 171 chars | description id 0cc8b2ca0aad
@@ -2776,103 +2860,102 @@
 "Tier 2 -L2": "R+S - Playbook Review/Maintenance" | type TODO | priority NONE | owner record's Site Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 171 chars | description id 0cc8b2ca0aad</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M19" s="5" t="inlineStr">
         <is>
           <t>11 (7 Create task, 4 If/then branch)</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N19" s="5" t="inlineStr">
         <is>
           <t>Creates task(s): "R+S - Playbook Review/Maintenance". Branches on: Customer Tier, Company name, Operations Manager, Site Manager</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O19" s="5" t="inlineStr">
         <is>
           <t>None (switched off as expected); titles: R+S - Playbook Review/Maintenance</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr">
+      <c r="P19" s="5" t="inlineStr">
         <is>
           <t>no queue on all 7 task action(s)</t>
         </is>
       </c>
-      <c r="Q20" s="5" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="R20" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-05 18:17:06 UTC</t>
-        </is>
-      </c>
-      <c r="S20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:23:04 UTC</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Create Tasks | Prepare Month End Report</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>1682101413</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Switched off. Would create monthly 'Prepare Month End Report' tasks.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Re-checked every month on day(s) 1 at 00:00</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "T2-L1 OM" if Operations Manager is known; "T2-L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K20" s="5" t="inlineStr">
         <is>
           <t>"Enterprise" &gt; "Enterprise OM": "R+S - Prepare Month End Report" | type TODO | priority NONE | owner record's Operations Manager | due 5 business day(s) after creation at 08:00 | queue Ops Tasks (13519269) | links Company = enrolled record | description 581 chars | description id 55dca87336ae
 "Enterprise" &gt; "Enterprise SM": "R+S - Prepare Month End Report" | type TODO | priority NONE | owner record's Site Manager | due 5 business day(s) after creation at 08:00 | queue Ops Tasks (13519269) | links Company = enrolled record | description 581 chars | description id 55dca87336ae
@@ -2884,104 +2967,102 @@
 "Tier 3": "R+S - Prepare Month End Report" | type TODO | priority NONE | owner record's Site Manager | due 5 business day(s) after creation at 08:00 | queue Ops Tasks (13519269) | links Company = enrolled record | description 581 chars | description id 55dca87336ae</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
         <is>
           <t>12 (8 Create task, 4 If/then branch)</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="N20" s="5" t="inlineStr">
         <is>
           <t>Creates task(s): "R+S - Prepare Month End Report"; "R+ S - Prepare Month End Report". Branches on: Customer Tier, Company name, Operations Manager, Site Manager</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
         <is>
           <t>None (switched off as expected); titles: R+S - Prepare Month End Report, R+ S - Prepare Month End Report</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr">
+      <c r="P20" s="5" t="inlineStr">
         <is>
           <t>Ops Tasks (13519269) on all 8 task action(s)</t>
         </is>
       </c>
-      <c r="Q21" s="5" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
-      <c r="R21" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-06 13:20:56 UTC</t>
-        </is>
-      </c>
-      <c r="S21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:15:32 UTC</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Create Tasks | Prepare Rate Review</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>1682549368</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Switched off. Would create weekly 'Prepare Rate Review' tasks.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Re-checked every week on monday at 00:00</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>record is in list 4291 "Exclude from Ops tasks"</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; "SOA" if Company name starts with SOA - ; otherwise end
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name doesn't contain exactly SOA; otherwise end
 At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
 At "Tier 1": "T1 OM" if Operations Manager is known; "T1 SM" if Site Manager is known; otherwise end
 At "Tier 2 - L1": "T2 - L1 OM" if Operations Manager is known; "T2 - L1 SM" if Site Manager is known; otherwise end
 "Enterprise" &gt; None met: ends with no task
 "Tier 1" &gt; None met: ends with no task
 "Tier 2 - L1" &gt; None met: ends with no task
-"Tier 2 - L2": ends with no task
-"SOA": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>"Enterprise" &gt; "Enterprise OM": "R+S - Prepare Rate Review" | type TODO | priority NONE | owner record's Operations Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 473 chars | description id 568c0ce68ef6
 "Enterprise" &gt; "Enterprise OM": "R+S - Prepare Rate Review" | type TODO | priority NONE | owner record's Operations Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 475 chars | description id 7c8a8a081da7
@@ -2999,7 +3080,7 @@
 "Tier 3": "R+S - Prepare Rate Review" | type TODO | priority NONE | owner record's Site Manager | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 471 chars | description id d119c3853ff9</t>
         </is>
       </c>
-      <c r="L22" s="5" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>"Enterprise" &gt; "Enterprise OM": Delay - 20160 minutes
 "Enterprise" &gt; "Enterprise OM": Delay - 15840 minutes
@@ -3017,99 +3098,93 @@
 "Tier 3": Delay - 25920 minutes</t>
         </is>
       </c>
-      <c r="M22" s="5" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>32 (14 Delay, 14 Create task, 4 If/then branch)</t>
         </is>
       </c>
-      <c r="N22" s="5" t="inlineStr">
+      <c r="N21" s="5" t="inlineStr">
         <is>
           <t>Creates task(s): "R+S - Prepare Rate Review"; "R+ S: Prepare Rate Review". Branches on: Customer Tier, Company name, Operations Manager, Site Manager</t>
         </is>
       </c>
-      <c r="O22" s="5" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>None (switched off as expected); titles: R+S - Prepare Rate Review, R+ S: Prepare Rate Review</t>
         </is>
       </c>
-      <c r="P22" s="5" t="inlineStr">
+      <c r="P21" s="5" t="inlineStr">
         <is>
           <t>no queue on all 14 task action(s)</t>
         </is>
       </c>
-      <c r="Q22" s="5" t="inlineStr">
-        <is>
-          <t>141</t>
-        </is>
-      </c>
-      <c r="R22" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-17 10:44:12 UTC</t>
-        </is>
-      </c>
-      <c r="S22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:25:12 UTC</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Create Tasks | Storage Reach</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>1697631666</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Switched off. Would create a weekly 'Storage Reach' task for fixed users.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Filter-based: Status is any of Live AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Re-checked every week on wednesday at 10:00</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Re-enroll ON; unenroll if no longer meets trigger OFF</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>record is in list 4291 "Exclude from Ops tasks"</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>At (start): "Enterprise" if Customer Tier is any of Enterprise AND Company name doesn't contain exactly SOA; "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 2 - L2" if Customer Tier is any of Tier 2 - L2 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name is equal to SOA; "SOA" if Company name starts with SOA - ; otherwise end
-At "Enterprise": "Enterprise OM" if Operations Manager is known; "Enterprise SM" if Site Manager is known; otherwise end
-At "Tier 1": "Is OM" if Operations Manager is known; "Is SM" if Site Manager is known; otherwise end
-"Enterprise" &gt; "Enterprise OM": ends with no task
-"Enterprise" &gt; "Enterprise SM": ends with no task
-"Enterprise" &gt; None met: ends with no task
-"Tier 1" &gt; "Is OM": ends with no task
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>At (start): "Tier 1" if Customer Tier is any of Tier 1 AND Company name doesn't contain exactly SOA; "Tier 2 - L1" if Customer Tier is any of Tier 2 - L1 AND Company name doesn't contain exactly SOA; "Tier 3" if Customer Tier is any of Tier 3 AND Company name is equal to SOA; "SOA" if Company name starts with SOA - ; otherwise end
+At "Tier 1": "Is SM" if Site Manager is known; otherwise end
 "Tier 1" &gt; None met: ends with no task
-"Tier 2 - L2": ends with no task
 None met: ends with no task</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
         <is>
           <t>"Tier 1" &gt; "Is SM": "R + S: Storage Reach" | type TODO | priority NONE | owner Kara Slavens (fixed user) | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 185 chars | description id d6ceb4006068
 "Tier 2 - L1": "R + S: Storage Reach" | type TODO | priority NONE | owner Hunter Stoner (fixed user) | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 185 chars | description id d6ceb4006068
@@ -3117,6 +3192,99 @@
 "SOA": "R+ S: Storage Reach" | type TODO | priority NONE | owner Luann Laughlin (fixed user) | due 2 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 185 chars | description id d6ceb4006068</t>
         </is>
       </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>6 (4 Create task, 2 If/then branch)</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>Creates task(s): "R + S: Storage Reach"; "R+ S: Storage Reach". Branches on: Customer Tier, Company name, Site Manager</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>None (switched off as expected); titles: R + S: Storage Reach, R+ S: Storage Reach</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>no queue on all 4 task action(s)</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:23:54 UTC</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>OM | RISK within the first 90 days</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>1774165521</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Switched off. Would create a task for the Operations Manager when a facility is At-Risk in its first 90 days.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Filter-based: Customer Health Score status is any of At-Risk AND Go Live Date is between today -90 days and now AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Re-enroll OFF; unenroll if no longer meets trigger OFF</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>record is in list 4291 "Exclude from Ops tasks"</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>(start): "" | type TODO | priority HIGH | owner record's Operations Manager | due 3 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 0 chars | description id da39a3ee5e6b</t>
+        </is>
+      </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
           <t>None</t>
@@ -3124,131 +3292,38 @@
       </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>7 (4 Create task, 3 If/then branch)</t>
+          <t>1 (1 Create task)</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Creates task(s): "R + S: Storage Reach"; "R+ S: Storage Reach". Branches on: Customer Tier, Company name, Operations Manager, Site Manager</t>
+          <t>No actions that create or change anything</t>
         </is>
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
-          <t>None (switched off as expected); titles: R + S: Storage Reach, R+ S: Storage Reach</t>
+          <t xml:space="preserve">None (switched off as expected); titles: </t>
         </is>
       </c>
       <c r="P23" s="5" t="inlineStr">
         <is>
-          <t>no queue on all 4 task action(s)</t>
+          <t>no queue on all 1 task action(s)</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R23" s="5" t="inlineStr">
         <is>
-          <t>2026-08-17 10:47:03 UTC</t>
+          <t>2026-08-17 10:41:58 UTC</t>
         </is>
       </c>
       <c r="S23" s="5" t="inlineStr"/>
     </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>OM | RISK within the first 90 days</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>1774165521</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>OFF</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Switched off. Would create a task for the Operations Manager when a facility is At-Risk in its first 90 days.</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Filter-based: Customer Health Score status is any of At-Risk AND Go Live Date is between today -90 days and now AND Full Management Type is any of Full management (Excl Call center), Full management (Incl Call center)</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Re-enroll OFF; unenroll if no longer meets trigger OFF</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>record is in list 4291 "Exclude from Ops tasks"</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>(start): "" | type TODO | priority HIGH | owner record's Operations Manager | due 3 business day(s) after creation at 08:00 | queue no queue | links Company = enrolled record | description 0 chars | description id da39a3ee5e6b</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
-        <is>
-          <t>1 (1 Create task)</t>
-        </is>
-      </c>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>No actions that create or change anything</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">None (switched off as expected); titles: </t>
-        </is>
-      </c>
-      <c r="P24" s="5" t="inlineStr">
-        <is>
-          <t>no queue on all 1 task action(s)</t>
-        </is>
-      </c>
-      <c r="Q24" s="5" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="R24" s="5" t="inlineStr">
-        <is>
-          <t>2026-08-17 10:41:58 UTC</t>
-        </is>
-      </c>
-      <c r="S24" s="5" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S24"/>
+  <autoFilter ref="A1:S23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3259,7 +3334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3294,7 +3369,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"2"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"6"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"5"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"2","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"3"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"3","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"4","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"5","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"6","listBranches":[{"branchName":"Tier 1 OM","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 1 SM","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L2 SM","connection":{"edgeType":"STANDARD","nextActionId":"4"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"12","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"NUMBER","operator":"IS_LESS_THAN","value":6.0},"property":"nps_customer_service_score"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"nps_customer_service_score"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1770961042","isEnabled":true,"name":"Create Tasks |  NPS Detractor Recovery Actions","objectTypeId":"0-2","revisionId":"54","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:23:05.897Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"2"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"6"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"5"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"2","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"3"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"3","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"4","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"5","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"6","listBranches":[{"branchName":"Tier 1 OM","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 1 SM","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L2 SM","connection":{"edgeType":"STANDARD","nextActionId":"4"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"12","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":717,"_sha1":"6dc3115f7d2b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":" NPS Detractor Recovery Actions","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"NUMBER","operator":"IS_LESS_THAN","value":6.0},"property":"nps_customer_service_score"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"nps_customer_service_score"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1770961042","isEnabled":true,"name":"Create Tasks |  NPS Detractor Recovery Actions","objectTypeId":"0-2","revisionId":"55","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:15:10.161Z"}</t>
         </is>
       </c>
     </row>
@@ -3309,7 +3384,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"4"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"3"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA -"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"2","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"3","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"2"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"4","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"6"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"6","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"7","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["WEDNESDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1770960918","isEnabled":true,"name":"Create Tasks | BOG Oversight Ent and T1","objectTypeId":"0-2","revisionId":"34","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:18:49.790Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"4"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"3"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"2","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"3","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"2"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"4","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"6"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"6","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"7","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":354,"_sha1":"e71a1efcf4ff"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"BOG Oversight","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["WEDNESDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1770960918","isEnabled":true,"name":"Create Tasks | BOG Oversight Ent and T1","objectTypeId":"0-2","revisionId":"36","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:16:15.653Z"}</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3399,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":496,"_sha1":"7136e41c55d6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts\n","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[25],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1838568063","isEnabled":true,"name":"Create Tasks | Confirm contacts on facility are correct","objectTypeId":"0-2","revisionId":"30","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:13:17.935Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":496,"_sha1":"7136e41c55d6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts\n","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":497,"_sha1":"78b156727ea8"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":500,"_sha1":"a1061918eebd"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Review Facility Contacts","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[25],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1838568063","isEnabled":true,"name":"Create Tasks | Confirm contacts on facility are correct","objectTypeId":"0-2","revisionId":"32","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:17:04.657Z"}</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3414,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"24"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Monthly Staus Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"16","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","listBranches":[{"branchName":"T2-L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2-L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"28800","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[10,20],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682560327","isEnabled":true,"name":"Create Tasks | Month End Call","objectTypeId":"0-2","revisionId":"103","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T10:36:59.329Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"24"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Monthly Staus Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"16","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","listBranches":[{"branchName":"T2-L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2-L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Bi-Weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":200,"_sha1":"537b9d134917"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Bi-weekly Call","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"28800","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[10,20],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682560327","isEnabled":true,"name":"Create Tasks | Month End Call","objectTypeId":"0-2","revisionId":"105","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:22:28.107Z"}</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3444,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"38"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"29"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"48"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"29","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"30","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"38","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"44"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"52"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"30"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"40","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"44","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"48","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise","TIER 2","TIER 1"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[2,17],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682542430","isEnabled":true,"name":"Create Tasks | Rate Review - Execution ENT, Tier 1 and Tier 2.1","objectTypeId":"0-2","revisionId":"140","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-06T11:01:53.441Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"38"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"29"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"48"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"29","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"30","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"38","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"44"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"52"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"30"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"40","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"44","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"48","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Rate Review - Execution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise","TIER 2","TIER 1"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[2,17],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682542430","isEnabled":true,"name":"Create Tasks | Rate Review - Execution ENT, Tier 1 and Tier 2.1","objectTypeId":"0-2","revisionId":"141","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-08T08:19:10.017Z"}</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3459,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"56"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"31"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"31","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Rate Review - Extecution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"56","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Rate Review - Extecution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2","TIER 3"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[15],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1868006300","isEnabled":true,"name":"Create Tasks | Rate Review - Execution Tier 2.2 and Tier 3","objectTypeId":"0-2","revisionId":"13","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-06T10:58:00.756Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"56"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"31"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"31","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Rate Review - Extecution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"56","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":140,"_sha1":"4423a979d75a"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Rate Review - Extecution","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2","TIER 3"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[15],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1868006300","isEnabled":true,"name":"Create Tasks | Rate Review - Execution Tier 2.2 and Tier 3","objectTypeId":"0-2","revisionId":"14","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-08T08:19:36.178Z"}</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3474,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"GOTO","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"cc7de124b1ad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":452,"_sha1":"7b79172f0612"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"798bffdcdfc2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, and SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"GOTO","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"798bffdcdfc2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, and SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"GOTO","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"cc7de124b1ad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1838565797","isEnabled":true,"name":"Create Tasks | Review Tow and Unsold Auctions report, action as needed","objectTypeId":"0-2","revisionId":"35","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T10:54:11.914Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"GOTO","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"cc7de124b1ad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":452,"_sha1":"7b79172f0612"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"798bffdcdfc2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, and SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"GOTO","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"798bffdcdfc2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, and SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"GOTO","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":454,"_sha1":"cc7de124b1ad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":10,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Unsold Unit, Towing, SCRA","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1838565797","isEnabled":true,"name":"Create Tasks | Review Tow and Unsold Auctions report, action as needed","objectTypeId":"0-2","revisionId":"36","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:20:19.412Z"}</t>
         </is>
       </c>
     </row>
@@ -3414,7 +3489,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_NONE_OF","values":["false"]},"property":"ppc_ads__yes_no_"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[6],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682548292","isEnabled":true,"name":"Create Tasks | Send Monthly Marketing Report Owner","objectTypeId":"0-2","revisionId":"90","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:24:49.663Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":269,"_sha1":"3bf5ebf7e8b2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S - Send Monthly Marketing Report to Owner","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_NONE_OF","values":["false"]},"property":"ppc_ads__yes_no_"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[6],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682548292","isEnabled":true,"name":"Create Tasks | Send Monthly Marketing Report Owner","objectTypeId":"0-2","revisionId":"91","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:14:43.282Z"}</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3504,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"36"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"37"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"12","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"27"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"27","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"36","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"46"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"37","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"46","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise","TIER 2","TIER 1"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[10],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682559152","isEnabled":true,"name":"Create Tasks | Update Customer Sentiment | Ent, Tier 1, Tier 2.1","objectTypeId":"0-2","revisionId":"142","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:10:58.618Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"36"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"37"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"12","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"27"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"27","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"36","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"46"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"37","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R + S- Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"46","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise","TIER 2","TIER 1"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[10],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682559152","isEnabled":true,"name":"Create Tasks | Update Customer Sentiment | Ent, Tier 1, Tier 2.1","objectTypeId":"0-2","revisionId":"145","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:17:52.621Z"}</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3519,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"52"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"29"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"29","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2","TIER 3"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[25],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1868006311","isEnabled":true,"name":"Create Tasks | Update Customer Sentiment |Tier 2.2, Tier 3","objectTypeId":"0-2","revisionId":"14","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:06:35.209Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"52"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"29"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"29","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":153,"_sha1":"5495b7a931eb"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Update Customer Sentiment","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2","TIER 3"]},"property":"customer_tier"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[25],"timeOfDay":{"hour":17,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1868006311","isEnabled":true,"name":"Create Tasks | Update Customer Sentiment |Tier 2.2, Tier 3","objectTypeId":"0-2","revisionId":"15","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:18:24.141Z"}</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3534,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days go live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"IS_NOT_EQUAL_TO","values":["Pinetop Self Storage"]},"property":"name"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838565644","isEnabled":true,"name":"Create Tasks | Weekly calls first 90 days after go live","objectTypeId":"0-2","revisionId":"39","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:15:48.937Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days go live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":264,"_sha1":"98833ac99ad9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"IS_NOT_EQUAL_TO","values":["Pinetop Self Storage"]},"property":"name"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838565644","isEnabled":true,"name":"Create Tasks | Weekly calls first 90 days after go live","objectTypeId":"0-2","revisionId":"43","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:12:55.261Z"}</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3549,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":151,"_sha1":"e34178af8de2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838568062","isEnabled":true,"name":"Create Tasks | Weekly KPI review to owner for first 90 days","objectTypeId":"0-2","revisionId":"28","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:17:37.031Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":151,"_sha1":"e34178af8de2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838568062","isEnabled":true,"name":"Create Tasks | Weekly KPI review to owner for first 90 days","objectTypeId":"0-2","revisionId":"32","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:12:20.649Z"}</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3564,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":513,"_sha1":"70ac668633b7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien Process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":350,"_sha1":"f6f59fb9e830"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":350,"_sha1":"f6f59fb9e830"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688964146","isEnabled":true,"name":"R+S - AI Lien Process","objectTypeId":"0-2","revisionId":"75","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:26:04.863Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":513,"_sha1":"70ac668633b7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien Process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":350,"_sha1":"f6f59fb9e830"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":350,"_sha1":"f6f59fb9e830"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":15,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - AI Lien process","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688964146","isEnabled":true,"name":"R+S - AI Lien Process","objectTypeId":"0-2","revisionId":"76","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:14:12.300Z"}</t>
         </is>
       </c>
     </row>
@@ -3519,14 +3594,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":385,"_sha1":"383c0c8de496"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"12","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"16","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":205,"_sha1":"5cff0ab1ea06"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688976731","isEnabled":true,"name":"R+S - Facility Performance Monitoring and Escalation","objectTypeId":"0-2","revisionId":"83","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:29:34.954Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":385,"_sha1":"383c0c8de496"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"12","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"16","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":205,"_sha1":"5cff0ab1ea06"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":384,"_sha1":"9343ddb3245c"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":7,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Facility Performance Monitoring and  Escalation","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688976731","isEnabled":true,"name":"R+S - Facility Performance Monitoring and Escalation","objectTypeId":"0-2","revisionId":"85","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:13:30.195Z"}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1689020435</t>
+          <t>1688833555</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3534,14 +3609,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"7"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"7","listBranches":[{"branchName":"T1 OM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"14","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"15"},"fields":{"delta":"1440","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"15","defaultBranchName":"SLA Met","listBranches":[{"branchName":"SLA not met","connection":{"edgeType":"STANDARD","nextActionId":"1"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"endpointBehavior":"EXCLUSIVE","includeObjectsWithNoValueSet":false,"operationType":"TIME_POINT","operator":"IS_BEFORE","propertyParser":"VALUE","timePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-1},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"type":"TIME_POINT"},"property":"notes_last_contacted"}]}],"filters":[]}}],"type":"LIST_BRANCH"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":185,"filterBranchOperator":"AND","filterBranchType":"ASSOCIATION","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["INCOMING_EMAIL"]},"property":"hs_email_direction"}],"objectTypeId":"0-49","operator":"IN_LIST"}],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1689020435","isEnabled":true,"name":"R+S - Reminders: Respond within 1 day to external emails","objectTypeId":"0-2","revisionId":"27","startActionId":"14","timeWindows":[],"updatedAt":"2026-10-06T13:26:35.902Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":139,"_sha1":"863f62f78287"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Execute Monthly Walk Through","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688833555","isEnabled":true,"name":"T1 SM SOA | R+S - Execute Monthly Walk Through - BOG","objectTypeId":"0-2","revisionId":"23","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:28:00.381Z"}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1688833555</t>
+          <t>1682545542</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3549,14 +3624,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"13"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"13","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":139,"_sha1":"863f62f78287"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Execute Monthly Walk Through","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1688833555","isEnabled":true,"name":"T1 SM SOA | R+S - Execute Monthly Walk Through - BOG","objectTypeId":"0-2","revisionId":"23","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:28:00.381Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 -L1","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 -L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1  SM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"21","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682545542","isEnabled":false,"name":"Create Tasks | Playbook Review/Maintenance T1 OM","objectTypeId":"0-2","revisionId":"66","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-08T08:23:04.163Z"}</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1682545542</t>
+          <t>1682101413</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3564,14 +3639,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 -L1","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 -L2","connection":{"edgeType":"STANDARD","nextActionId":"26"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1  SM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"21","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"26","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":171,"_sha1":"0cc8b2ca0aad"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Playbook Review/Maintenance","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":10,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682545542","isEnabled":false,"name":"Create Tasks | Playbook Review/Maintenance T1 OM","objectTypeId":"0-2","revisionId":"65","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-05T18:17:06.888Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"8","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"16","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"17","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"8"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","listBranches":[{"branchName":"T2-L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2-L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682101413","isEnabled":false,"name":"Create Tasks | Prepare Month End Report","objectTypeId":"0-2","revisionId":"109","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:15:32.574Z"}</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1682101413</t>
+          <t>1682549368</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3579,14 +3654,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"16"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"8","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"14","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"16","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"22"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"17","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"8"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"18","listBranches":[{"branchName":"T2-L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2-L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"14"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"19","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"22","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":581,"_sha1":"55dca87336ae"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":5,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"R+ S - Prepare Month End Report","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfMonth":[1],"timeOfDay":{"hour":0,"minute":0},"type":"MONTHLY_SPECIFIC_DAYS"},"id":"1682101413","isEnabled":false,"name":"Create Tasks | Prepare Month End Report","objectTypeId":"0-2","revisionId":"108","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-06T13:20:56.435Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"41"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"32"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"12","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"30"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"54"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"16","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"34"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"35"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"36"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"30","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"16"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"31","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"20"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"32","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"23"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":471,"_sha1":"d119c3853ff9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"34","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"38"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"35","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"39"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"36","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"37"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":471,"_sha1":"d119c3853ff9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"37","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"38","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"39","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"40","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"46"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"50"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"41","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"31"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"43"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"43","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"44"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"44","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"45"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"45","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"46","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"47"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"47","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"48"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"48","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"49"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"49","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"50","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"51"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"51","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"52"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"53"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"53","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"54","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"55"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"55","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"56"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"56","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"57"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"57","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":0,"minute":0},"type":"WEEKLY"},"id":"1682549368","isEnabled":false,"name":"Create Tasks | Prepare Rate Review","objectTypeId":"0-2","revisionId":"142","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-08T08:25:12.331Z"}</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1682549368</t>
+          <t>1697631666</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -3594,35 +3669,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"12"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"41"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"32"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"12","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"30"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T1 SM","connection":{"edgeType":"STANDARD","nextActionId":"54"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"16","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"34"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"20","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"35"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"23","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"36"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"30","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"16"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"31","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"20"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"32","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"23"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":471,"_sha1":"d119c3853ff9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"34","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"38"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"35","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"39"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"36","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"37"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":471,"_sha1":"d119c3853ff9"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"37","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"38","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"39","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"40","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"46"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"50"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"41","listBranches":[{"branchName":"T2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"T2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"31"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"43"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"43","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"44"},"fields":{"delta":"30240","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"44","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"45"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"fd4557e25325"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+ S: Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"45","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"25920","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"46","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"47"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"47","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"48"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"48","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"49"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"49","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"50","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"51"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"51","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"52"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"52","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"53"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"53","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"54","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"55"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":473,"_sha1":"568c0ce68ef6"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"55","actionTypeId":"0-1","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"56"},"fields":{"delta":"20160","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"},{"actionId":"56","actionTypeId":"0-3","actionTypeVersion":0,"connection":{"edgeType":"STANDARD","nextActionId":"57"},"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":475,"_sha1":"7c8a8a081da7"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","subject":"R+S - Prepare Rate Review","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"57","actionTypeId":"0-1","actionTypeVersion":0,"fields":{"delta":"15840","time_unit":"MINUTES"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":0,"minute":0},"type":"WEEKLY"},"id":"1682549368","isEnabled":false,"name":"Create Tasks | Prepare Rate Review","objectTypeId":"0-2","revisionId":"141","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-08-17T10:44:12.978Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"38"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"41"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"IS_EQUAL_TO","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"38","listBranches":[{"branchName":"Is SM","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"80578237","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"40","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"80038421","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"41","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"845242816","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"81572740","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R+ S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["WEDNESDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1697631666","isEnabled":false,"name":"Create Tasks | Storage Reach","objectTypeId":"0-2","revisionId":"23","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-10-08T08:23:54.611Z"}</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1697631666</t>
+          <t>1774165521</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="inlineStr">
-        <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"43"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"38"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"40"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"41"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"IS_EQUAL_TO","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"SOA","connection":{"edgeType":"STANDARD","nextActionId":"42"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"STARTS_WITH","values":["SOA - "]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"38","listBranches":[{"branchName":"Is OM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Is SM","connection":{"edgeType":"STANDARD","nextActionId":"39"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"39","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"80578237","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"40","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"80038421","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"41","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"845242816","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R + S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"42","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":185,"_sha1":"d6ceb4006068"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"staticValue":"81572740","type":"STATIC_VALUE"}},"priority":"NONE","subject":"R+ S: Storage Reach","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"43","listBranches":[{"branchName":"Enterprise OM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Yes"]},"property":"live"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["WEDNESDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1697631666","isEnabled":false,"name":"Create Tasks | Storage Reach","objectTypeId":"0-2","revisionId":"21","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-08-17T10:47:03.705Z"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>1774165521</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" t="inlineStr">
         <is>
           <t>{"actions":[{"actionId":"1","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":0,"_sha1":"da39a3ee5e6b"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":3,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"HIGH","subject":"","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["At-Risk"]},"property":"customer_health_score_status"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-90},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":false,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"id":"1774165521","isEnabled":false,"name":"OM | RISK within the first 90 days","objectTypeId":"0-2","revisionId":"8","startActionId":"1","suppressionFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"IN_LIST","listId":"4291","operator":"IN_LIST"}]}],"filters":[]},"timeWindows":[],"updatedAt":"2026-08-17T10:41:58.087Z"}</t>
         </is>

</xml_diff>

<commit_message>
CS Ops: Weekly KPI review switched off as planned (duplicate of Weekly calls, confirmed by Cherine); master rules file updated and logged; Waiting on Cherine item 2 closed; Switched off summary added
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TuFPqtNuPi7KBKeykeDCDb
</commit_message>
<xml_diff>
--- a/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
+++ b/audits/cs-ops-workflow-audit/CS_Ops_Master_Rules.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -902,6 +902,18 @@
       <c r="B37" s="3" t="inlineStr">
         <is>
           <t>2026-10-08: removed R+S - Reminders: Respond within 1 day to external emails (1689020435). Deleted in HubSpot on purpose (confirmed by WLS on 2026-10-08); the API now returns 404. Closes known issue F-05 and Waiting on Cherine item 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Change log</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-08: updated 1838568062. Planned (confirmed by Cherine on 2026-10-08): switched off as the duplicate of Create Tasks | Weekly calls first 90 days after go live. Revision 32 -&gt; 33, switched off 2026-10-08 09:37 UTC. Closes Waiting on Cherine item 2.</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2310,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -2376,12 +2388,12 @@
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>2026-10-08 08:12:20 UTC</t>
+          <t>2026-10-08 09:37:28 UTC</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr"/>
@@ -3549,7 +3561,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":151,"_sha1":"e34178af8de2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838568062","isEnabled":true,"name":"Create Tasks | Weekly KPI review to owner for first 90 days","objectTypeId":"0-2","revisionId":"32","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T08:12:20.649Z"}</t>
+          <t>{"actions":[{"actionId":"1","listBranches":[{"branchName":"Enterprise","connection":{"edgeType":"STANDARD","nextActionId":"19"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Enterprise"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 1","connection":{"edgeType":"STANDARD","nextActionId":"11"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 1"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L1","connection":{"edgeType":"STANDARD","nextActionId":"23"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 2 - L2","connection":{"edgeType":"STANDARD","nextActionId":"25"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Tier 2 - L2"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}},{"branchName":"Tier 3","connection":{"edgeType":"STANDARD","nextActionId":"18"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["TIER 3"]},"property":"customer_tier"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"MULTISTRING","operator":"DOES_NOT_CONTAIN_EXACTLY","values":["SOA"]},"property":"name"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"11","listBranches":[{"branchName":"T1 OM","connection":{"edgeType":"STANDARD","nextActionId":"15"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"15","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"17","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"18","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":151,"_sha1":"e34178af8de2"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"19","listBranches":[{"branchName":"Enterprise OM","connection":{"edgeType":"STANDARD","nextActionId":"20"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Enterprise SM","connection":{"edgeType":"STANDARD","nextActionId":"21"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"20","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"21","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly KPI Review: First 90 days live","task_type":"TODO","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"23","listBranches":[{"branchName":"Tier 2 - L1 OM","connection":{"edgeType":"STANDARD","nextActionId":"24"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"operations_manager"}]}],"filters":[]}},{"branchName":"Tier 2 - L1 SM","connection":{"edgeType":"STANDARD","nextActionId":"17"},"filterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ALL_PROPERTY","operator":"IS_KNOWN"},"property":"site_manager"}]}],"filters":[]}}],"type":"LIST_BRANCH"},{"actionId":"24","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"operations_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"},{"actionId":"25","actionTypeId":"0-3","actionTypeVersion":0,"fields":{"associations":[{"target":{"associationCategory":"HUBSPOT_DEFINED","associationTypeId":192},"value":{"type":"ENROLLED_OBJECT"}}],"body":{"_len":113,"_sha1":"c10c1946e350"},"due_time":{"daysOfWeek":["MONDAY","TUESDAY","WEDNESDAY","THURSDAY","FRIDAY"],"delta":2,"timeOfDay":{"hour":8,"minute":0},"timeUnit":"DAYS"},"owner_assignment":{"type":"CUSTOM","value":{"propertyName":"site_manager","type":"OBJECT_PROPERTY"}},"priority":"NONE","queue_id":"13519269","subject":"Weekly Call: First 90 days Live\n","task_type":"CALL","use_explicit_associations":"true"},"type":"SINGLE_CONNECTION"}],"blockedDates":[],"enrollmentCriteria":{"listFilterBranch":{"filterBranchOperator":"OR","filterBranchType":"OR","filterBranches":[{"filterBranchOperator":"AND","filterBranchType":"AND","filterBranches":[],"filters":[{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"lowerBoundEndpointBehavior":"INCLUSIVE","lowerBoundTimePoint":{"indexReference":{"referenceType":"TODAY"},"offset":{"days":-91},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"},"operationType":"TIME_RANGED","operator":"IS_BETWEEN","propertyParser":"VALUE_WITH_ZONE_SAME_LOCAL_CONVERSION","type":"TIME_RANGED","upperBoundEndpointBehavior":"INCLUSIVE","upperBoundTimePoint":{"indexReference":{"referenceType":"NOW"},"timeType":"INDEXED","timezoneSource":"CUSTOM","zoneId":"US/Eastern"}},"property":"go_live_date"},{"filterType":"PROPERTY","operation":{"includeObjectsWithNoValueSet":false,"operationType":"ENUMERATION","operator":"IS_ANY_OF","values":["Full management (Excl Call center)","Full TPM"]},"property":"mgt_type"}]}],"filters":[]},"reEnrollmentTriggersFilterBranches":[],"shouldReEnroll":true,"type":"LIST_BASED","unEnrollObjectsNotMeetingCriteria":false},"enrollmentSchedule":{"daysOfWeek":["MONDAY"],"timeOfDay":{"hour":10,"minute":0},"type":"WEEKLY"},"id":"1838568062","isEnabled":false,"name":"Create Tasks | Weekly KPI review to owner for first 90 days","objectTypeId":"0-2","revisionId":"33","startActionId":"1","timeWindows":[],"updatedAt":"2026-10-08T09:37:28.842Z"}</t>
         </is>
       </c>
     </row>

</xml_diff>